<commit_message>
Gantt chart and journal updation
</commit_message>
<xml_diff>
--- a/docs/campus_connect-gantt-chart_ms.xlsx
+++ b/docs/campus_connect-gantt-chart_ms.xlsx
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="E3" s="55" t="n">
-        <v>46279</v>
+        <v>46306</v>
       </c>
       <c r="F3" s="53" t="n"/>
     </row>
@@ -4760,10 +4760,20 @@
           <t>Task 6.1 — Events API (src/app/api/events)</t>
         </is>
       </c>
-      <c r="C45" s="39" t="n"/>
-      <c r="D45" s="42" t="n"/>
-      <c r="E45" s="57" t="n"/>
-      <c r="F45" s="58" t="n"/>
+      <c r="C45" s="39" t="inlineStr">
+        <is>
+          <t>Aayushmaan Singh Meyan</t>
+        </is>
+      </c>
+      <c r="D45" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="57" t="n">
+        <v>46299</v>
+      </c>
+      <c r="F45" s="58" t="n">
+        <v>46300</v>
+      </c>
       <c r="G45" s="16" t="n"/>
       <c r="H45" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -4833,10 +4843,20 @@
           <t>Task 6.2 — Schedule UI (CalendarView &amp; EventModal)</t>
         </is>
       </c>
-      <c r="C46" s="39" t="n"/>
-      <c r="D46" s="42" t="n"/>
-      <c r="E46" s="57" t="n"/>
-      <c r="F46" s="58" t="n"/>
+      <c r="C46" s="39" t="inlineStr">
+        <is>
+          <t>Aayushmaan Singh Meyan</t>
+        </is>
+      </c>
+      <c r="D46" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="57" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F46" s="58" t="n">
+        <v>46301</v>
+      </c>
       <c r="G46" s="16" t="n"/>
       <c r="H46" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -4906,10 +4926,20 @@
           <t>Task 6.3 — Event Notifications &amp; Socket Broadcast</t>
         </is>
       </c>
-      <c r="C47" s="39" t="n"/>
-      <c r="D47" s="42" t="n"/>
-      <c r="E47" s="57" t="n"/>
-      <c r="F47" s="58" t="n"/>
+      <c r="C47" s="39" t="inlineStr">
+        <is>
+          <t>Aayushmaan Singh Meyan</t>
+        </is>
+      </c>
+      <c r="D47" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="57" t="n">
+        <v>46301</v>
+      </c>
+      <c r="F47" s="58" t="n">
+        <v>46301</v>
+      </c>
       <c r="G47" s="16" t="n"/>
       <c r="H47" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5052,10 +5082,20 @@
           <t>Task 7.1 — Custom Server Setup (server.ts with Socket.io)</t>
         </is>
       </c>
-      <c r="C49" s="39" t="n"/>
-      <c r="D49" s="42" t="n"/>
-      <c r="E49" s="57" t="n"/>
-      <c r="F49" s="58" t="n"/>
+      <c r="C49" s="39" t="inlineStr">
+        <is>
+          <t>Divyansh Jasrotia</t>
+        </is>
+      </c>
+      <c r="D49" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="57" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F49" s="58" t="n">
+        <v>46302</v>
+      </c>
       <c r="G49" s="16" t="n"/>
       <c r="H49" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5125,10 +5165,20 @@
           <t>Task 7.2 — Messaging API (src/app/api/messages)</t>
         </is>
       </c>
-      <c r="C50" s="39" t="n"/>
-      <c r="D50" s="42" t="n"/>
-      <c r="E50" s="57" t="n"/>
-      <c r="F50" s="58" t="n"/>
+      <c r="C50" s="39" t="inlineStr">
+        <is>
+          <t>Divyansh Jasrotia</t>
+        </is>
+      </c>
+      <c r="D50" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="57" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F50" s="58" t="n">
+        <v>46303</v>
+      </c>
       <c r="G50" s="16" t="n"/>
       <c r="H50" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5198,10 +5248,20 @@
           <t>Task 7.3 — Messaging UI (UserChatList &amp; ChatBox)</t>
         </is>
       </c>
-      <c r="C51" s="39" t="n"/>
-      <c r="D51" s="42" t="n"/>
-      <c r="E51" s="57" t="n"/>
-      <c r="F51" s="58" t="n"/>
+      <c r="C51" s="39" t="inlineStr">
+        <is>
+          <t>Divyansh Jasrotia</t>
+        </is>
+      </c>
+      <c r="D51" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="57" t="n">
+        <v>46303</v>
+      </c>
+      <c r="F51" s="58" t="n">
+        <v>46304</v>
+      </c>
       <c r="G51" s="16" t="n"/>
       <c r="H51" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5271,10 +5331,20 @@
           <t>Task 7.4 — Notifications API (src/app/api/notifications)</t>
         </is>
       </c>
-      <c r="C52" s="39" t="n"/>
-      <c r="D52" s="42" t="n"/>
-      <c r="E52" s="57" t="n"/>
-      <c r="F52" s="58" t="n"/>
+      <c r="C52" s="39" t="inlineStr">
+        <is>
+          <t>Prakhar Saxena</t>
+        </is>
+      </c>
+      <c r="D52" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="57" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F52" s="58" t="n">
+        <v>46305</v>
+      </c>
       <c r="G52" s="16" t="n"/>
       <c r="H52" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5344,10 +5414,20 @@
           <t>Task 7.5 — Notification Bell UI (NotificationDropdown.tsx)</t>
         </is>
       </c>
-      <c r="C53" s="39" t="n"/>
-      <c r="D53" s="42" t="n"/>
-      <c r="E53" s="57" t="n"/>
-      <c r="F53" s="58" t="n"/>
+      <c r="C53" s="39" t="inlineStr">
+        <is>
+          <t>Prakhar Saxena</t>
+        </is>
+      </c>
+      <c r="D53" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="57" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F53" s="58" t="n">
+        <v>46305</v>
+      </c>
       <c r="G53" s="16" t="n"/>
       <c r="H53" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
@@ -5490,10 +5570,20 @@
           <t>Task 8.1 — Admin API Routes (Users, Settings, Reports)</t>
         </is>
       </c>
-      <c r="C55" s="39" t="n"/>
-      <c r="D55" s="42" t="n"/>
-      <c r="E55" s="57" t="n"/>
-      <c r="F55" s="58" t="n"/>
+      <c r="C55" s="39" t="inlineStr">
+        <is>
+          <t>Prakhar Saxena</t>
+        </is>
+      </c>
+      <c r="D55" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="57" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F55" s="58" t="n">
+        <v>46306</v>
+      </c>
       <c r="G55" s="16" t="n"/>
       <c r="H55" s="16">
         <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>

</xml_diff>